<commit_message>
teste integração com clp
</commit_message>
<xml_diff>
--- a/clp/qualidade/tagPrensa.xlsx
+++ b/clp/qualidade/tagPrensa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\hostLinkOmron\hotsLinkOmron\clp\qualidade\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA8E2E80-AD3C-4911-8F9A-0E38535D2B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB58C96F-D945-4487-9AF3-E5DE81D26DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1870" uniqueCount="706">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1874" uniqueCount="711">
   <si>
     <t>prensa29</t>
   </si>
@@ -2055,15 +2055,6 @@
     <t>Segundo</t>
   </si>
   <si>
-    <t>D321</t>
-  </si>
-  <si>
-    <t>D323</t>
-  </si>
-  <si>
-    <t>D325</t>
-  </si>
-  <si>
     <t>PONTEIRO INICIO</t>
   </si>
   <si>
@@ -2158,6 +2149,30 @@
   </si>
   <si>
     <t>minuto e segundo clp</t>
+  </si>
+  <si>
+    <t>D3002</t>
+  </si>
+  <si>
+    <t>D3003</t>
+  </si>
+  <si>
+    <t>D3004</t>
+  </si>
+  <si>
+    <t>D3005</t>
+  </si>
+  <si>
+    <t>D3006</t>
+  </si>
+  <si>
+    <t>D3001...D3006</t>
+  </si>
+  <si>
+    <t>D3007</t>
+  </si>
+  <si>
+    <t>D3008...D3007</t>
   </si>
 </sst>
 </file>
@@ -2242,9 +2257,6 @@
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2253,6 +2265,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2812,20 +2827,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="6" t="s">
         <v>531</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="H1" s="2" t="s">
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="H1" s="6" t="s">
         <v>530</v>
       </c>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -10990,8 +11005,8 @@
     <col min="4" max="4" width="20.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -11006,44 +11021,44 @@
       <c r="A2" t="s">
         <v>648</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>584</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>651</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>659</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="3" t="s">
         <v>663</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="3" t="s">
         <v>664</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>652</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>585</v>
       </c>
-      <c r="H4" s="5" t="s">
-        <v>590</v>
-      </c>
-      <c r="I4" s="5" t="s">
+      <c r="H4" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="I4" s="4" t="s">
         <v>665</v>
       </c>
     </row>
@@ -11051,16 +11066,16 @@
       <c r="A5" t="s">
         <v>653</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>660</v>
       </c>
-      <c r="H5" s="5" t="s">
-        <v>671</v>
-      </c>
-      <c r="I5" s="5" t="s">
+      <c r="H5" s="4" t="s">
+        <v>703</v>
+      </c>
+      <c r="I5" s="4" t="s">
         <v>666</v>
       </c>
     </row>
@@ -11068,16 +11083,16 @@
       <c r="A6" t="s">
         <v>654</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>586</v>
       </c>
-      <c r="H6" s="5" t="s">
-        <v>591</v>
-      </c>
-      <c r="I6" s="5" t="s">
+      <c r="H6" s="4" t="s">
+        <v>704</v>
+      </c>
+      <c r="I6" s="4" t="s">
         <v>667</v>
       </c>
     </row>
@@ -11085,62 +11100,62 @@
       <c r="A7" t="s">
         <v>655</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>661</v>
       </c>
-      <c r="H7" s="5" t="s">
-        <v>672</v>
-      </c>
-      <c r="I7" s="5" t="s">
+      <c r="H7" s="4" t="s">
+        <v>705</v>
+      </c>
+      <c r="I7" s="4" t="s">
         <v>668</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>674</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>675</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>592</v>
-      </c>
-      <c r="I8" s="5" t="s">
+        <v>671</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>672</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>706</v>
+      </c>
+      <c r="I8" s="4" t="s">
         <v>669</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>677</v>
-      </c>
-      <c r="C9" s="6" t="s">
+        <v>674</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>589</v>
       </c>
-      <c r="H9" s="5" t="s">
-        <v>673</v>
-      </c>
-      <c r="I9" s="5" t="s">
+      <c r="H9" s="4" t="s">
+        <v>707</v>
+      </c>
+      <c r="I9" s="4" t="s">
         <v>670</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="F11" t="s">
-        <v>676</v>
+        <v>673</v>
       </c>
       <c r="G11" t="s">
         <v>165</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="H11" s="4" t="s">
         <v>581</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I11" s="4" t="s">
         <v>656</v>
       </c>
       <c r="J11" t="s">
@@ -11154,28 +11169,28 @@
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2"/>
       <c r="F12" t="s">
-        <v>677</v>
+        <v>674</v>
       </c>
       <c r="G12" t="s">
         <v>589</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2"/>
       <c r="F13" t="s">
-        <v>678</v>
+        <v>675</v>
       </c>
       <c r="G13" t="s">
         <v>159</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="H13" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="I13" s="4" t="s">
         <v>581</v>
       </c>
       <c r="J13" t="s">
@@ -11189,48 +11204,62 @@
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
       <c r="F15" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
       <c r="G15" t="s">
-        <v>676</v>
+        <v>673</v>
       </c>
       <c r="H15" t="s">
+        <v>674</v>
+      </c>
+      <c r="I15" t="s">
         <v>677</v>
       </c>
-      <c r="I15" t="s">
-        <v>680</v>
-      </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
       <c r="F16" t="s">
         <v>159</v>
       </c>
       <c r="G16" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="H16" t="s">
         <v>658</v>
       </c>
       <c r="I16" t="s">
-        <v>682</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F17" t="s">
+        <v>162</v>
+      </c>
+      <c r="G17" t="s">
+        <v>708</v>
+      </c>
+      <c r="H17" t="s">
+        <v>709</v>
+      </c>
+      <c r="I17" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>692</v>
+        <v>689</v>
       </c>
       <c r="B23" t="s">
         <v>14</v>
@@ -11239,15 +11268,15 @@
         <v>165</v>
       </c>
       <c r="D23" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="E23">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>693</v>
+        <v>690</v>
       </c>
       <c r="B24" t="s">
         <v>14</v>
@@ -11256,15 +11285,15 @@
         <v>581</v>
       </c>
       <c r="D24" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
       <c r="E24">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>694</v>
+        <v>691</v>
       </c>
       <c r="B25" t="s">
         <v>14</v>
@@ -11273,15 +11302,15 @@
         <v>656</v>
       </c>
       <c r="D25" t="s">
-        <v>685</v>
+        <v>682</v>
       </c>
       <c r="E25">
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>695</v>
+        <v>692</v>
       </c>
       <c r="B26" t="s">
         <v>14</v>
@@ -11290,15 +11319,15 @@
         <v>582</v>
       </c>
       <c r="D26" t="s">
-        <v>686</v>
+        <v>683</v>
       </c>
       <c r="E26">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
       <c r="B27" t="s">
         <v>14</v>
@@ -11307,15 +11336,15 @@
         <v>657</v>
       </c>
       <c r="D27" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
       <c r="E27">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
       <c r="B28" t="s">
         <v>14</v>
@@ -11324,15 +11353,15 @@
         <v>583</v>
       </c>
       <c r="D28" t="s">
-        <v>688</v>
+        <v>685</v>
       </c>
       <c r="E28">
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
       <c r="B29" t="s">
         <v>14</v>
@@ -11341,58 +11370,58 @@
         <v>658</v>
       </c>
       <c r="D29" t="s">
-        <v>689</v>
+        <v>686</v>
       </c>
       <c r="E29">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>696</v>
+      </c>
+      <c r="B30" t="s">
+        <v>14</v>
+      </c>
+      <c r="C30" t="s">
+        <v>687</v>
+      </c>
+      <c r="D30" t="s">
+        <v>688</v>
+      </c>
+      <c r="E30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>699</v>
       </c>
-      <c r="B30" t="s">
-        <v>14</v>
-      </c>
-      <c r="C30" t="s">
-        <v>690</v>
-      </c>
-      <c r="D30" t="s">
-        <v>691</v>
-      </c>
-      <c r="E30">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="B31" t="s">
+        <v>14</v>
+      </c>
+      <c r="C31" t="s">
+        <v>697</v>
+      </c>
+      <c r="D31" t="s">
+        <v>698</v>
+      </c>
+      <c r="E31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>700</v>
+      </c>
+      <c r="B32" t="s">
+        <v>14</v>
+      </c>
+      <c r="C32" t="s">
+        <v>701</v>
+      </c>
+      <c r="D32" t="s">
         <v>702</v>
-      </c>
-      <c r="B31" t="s">
-        <v>14</v>
-      </c>
-      <c r="C31" t="s">
-        <v>700</v>
-      </c>
-      <c r="D31" t="s">
-        <v>701</v>
-      </c>
-      <c r="E31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>703</v>
-      </c>
-      <c r="B32" t="s">
-        <v>14</v>
-      </c>
-      <c r="C32" t="s">
-        <v>704</v>
-      </c>
-      <c r="D32" t="s">
-        <v>705</v>
       </c>
       <c r="E32">
         <v>0</v>

</xml_diff>